<commit_message>
Restore VITAL alcohol-RCC estimate to pooled results
</commit_message>
<xml_diff>
--- a/summary/no/exposures_meta_analysis_kidney_and_renal_pelvis_cancer_combined.xlsx
+++ b/summary/no/exposures_meta_analysis_kidney_and_renal_pelvis_cancer_combined.xlsx
@@ -450,7 +450,7 @@
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
-  <sheetData>
+  <sheetData xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
@@ -509,10 +509,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>selenium</t>
-        </is>
+      <c r="A2" t="str">
+        <v>selenium</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2</v>
@@ -526,12 +524,12 @@
       <c r="E2" s="3" t="n">
         <v>0.9175942312201509</v>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="4" t="n">
         <v>95.27</v>
       </c>
-      <c r="I2" s="5" t="inlineStr"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="2" t="n">
         <v>3471</v>
       </c>
@@ -540,10 +538,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>iron</t>
-        </is>
+      <c r="A3" t="str">
+        <v>iron</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1</v>
@@ -557,10 +553,10 @@
       <c r="E3" s="3" t="n">
         <v>0.6705760782100518</v>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="5"/>
       <c r="J3" s="2" t="n">
         <v>6109</v>
       </c>
@@ -569,10 +565,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>linoleic_acid</t>
-        </is>
+      <c r="A4" t="str">
+        <v>linoleic_acid</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>1</v>
@@ -586,10 +580,10 @@
       <c r="E4" s="3" t="n">
         <v>0.7010934955249702</v>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="5"/>
       <c r="J4" s="2" t="n">
         <v>2301</v>
       </c>
@@ -598,10 +592,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>tomato</t>
-        </is>
+      <c r="A5" t="str">
+        <v>tomato</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1</v>
@@ -615,10 +607,10 @@
       <c r="E5" s="3" t="n">
         <v>0.8108009172540728</v>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="5"/>
       <c r="J5" s="2" t="n">
         <v>672</v>
       </c>
@@ -627,10 +619,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>green_tea</t>
-        </is>
+      <c r="A6" t="str">
+        <v>green_tea</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2</v>
@@ -644,12 +634,12 @@
       <c r="E6" s="3" t="n">
         <v>1.109156703489818</v>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="4" t="n">
         <v>83.87</v>
       </c>
-      <c r="I6" s="5" t="inlineStr"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="2" t="n">
         <v>103012</v>
       </c>
@@ -658,10 +648,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>quercetin</t>
-        </is>
+      <c r="A7" t="str">
+        <v>quercetin</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>1</v>
@@ -675,10 +663,10 @@
       <c r="E7" s="3" t="n">
         <v>0.9002344022096688</v>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="5"/>
       <c r="J7" s="2" t="n">
         <v>27111</v>
       </c>
@@ -687,10 +675,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>plant_protein_intake</t>
-        </is>
+      <c r="A8" t="str">
+        <v>plant_protein_intake</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1</v>
@@ -704,10 +690,10 @@
       <c r="E8" s="3" t="n">
         <v>0.8104008904442759</v>
       </c>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="5"/>
       <c r="J8" s="2" t="n">
         <v>87841</v>
       </c>
@@ -716,10 +702,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>vitamin_b12</t>
-        </is>
+      <c r="A9" t="str">
+        <v>vitamin_b12</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>2</v>
@@ -733,12 +717,12 @@
       <c r="E9" s="3" t="n">
         <v>0.8542768136084795</v>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
       <c r="H9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I9" s="5" t="inlineStr"/>
+      <c r="I9" s="5"/>
       <c r="J9" s="2" t="n">
         <v>1959</v>
       </c>
@@ -747,10 +731,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>eggs</t>
-        </is>
+      <c r="A10" t="str">
+        <v>eggs</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1</v>
@@ -764,10 +746,10 @@
       <c r="E10" s="3" t="n">
         <v>0.8606264155428169</v>
       </c>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="5"/>
       <c r="J10" s="2" t="n">
         <v>1812</v>
       </c>
@@ -776,10 +758,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>folic_acid</t>
-        </is>
+      <c r="A11" t="str">
+        <v>folic_acid</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>6</v>
@@ -800,7 +780,7 @@
         <v>1.822081402776787</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>70.06999999999999</v>
+        <v>70.07</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0.2283849913275224</v>
@@ -813,10 +793,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>vitamin_e</t>
-        </is>
+      <c r="A12" t="str">
+        <v>vitamin_e</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>4</v>
@@ -837,7 +815,7 @@
         <v>3.723705085890995</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>75.48999999999999</v>
+        <v>75.49</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>0.498302423964353</v>
@@ -850,10 +828,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>anti_inflammatory_diet</t>
-        </is>
+      <c r="A13" t="str">
+        <v>anti_inflammatory_diet</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1</v>
@@ -867,10 +843,10 @@
       <c r="E13" s="3" t="n">
         <v>0.8902549819435438</v>
       </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="5"/>
       <c r="J13" s="2" t="n">
         <v>71421</v>
       </c>
@@ -879,10 +855,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>tea</t>
-        </is>
+      <c r="A14" t="str">
+        <v>tea</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>5</v>
@@ -916,10 +890,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>vitamin_b6</t>
-        </is>
+      <c r="A15" t="str">
+        <v>vitamin_b6</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>3</v>
@@ -953,10 +925,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>beta_carotene</t>
-        </is>
+      <c r="A16" t="str">
+        <v>beta_carotene</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>5</v>
@@ -990,10 +960,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>vitamin_c</t>
-        </is>
+      <c r="A17" t="str">
+        <v>vitamin_c</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>5</v>
@@ -1027,10 +995,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>pyridoxal_5_phosphate_plp</t>
-        </is>
+      <c r="A18" t="str">
+        <v>pyridoxal_5_phosphate_plp</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>1</v>
@@ -1044,10 +1010,10 @@
       <c r="E18" s="3" t="n">
         <v>0.8705884045850067</v>
       </c>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="5" t="inlineStr"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="5"/>
       <c r="J18" s="2" t="n">
         <v>910</v>
       </c>
@@ -1056,47 +1022,43 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>alcohol</t>
-        </is>
+      <c r="A19" t="str">
+        <v>alcohol</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0.76958797865763</v>
+        <v>0.7676664116705357</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.6985838950869678</v>
+        <v>0.6978158752907021</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.8478089189568343</v>
+        <v>0.8445089033860343</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0.5102524008301632</v>
+        <v>0.5102473715430387</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>1.160730759778378</v>
+        <v>1.154952974720829</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>79.11</v>
+        <v>78.51</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.007772801972821657</v>
+        <v>0.005921333962773998</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>14155769</v>
+        <v>14233029</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>29965</v>
+        <v>30214</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>lutein</t>
-        </is>
+      <c r="A20" t="str">
+        <v>lutein</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>5</v>
@@ -1130,10 +1092,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>betaine</t>
-        </is>
+      <c r="A21" t="str">
+        <v>betaine</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>1</v>
@@ -1147,10 +1107,10 @@
       <c r="E21" s="3" t="n">
         <v>1.24</v>
       </c>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="5" t="inlineStr"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="5"/>
       <c r="J21" s="2" t="n">
         <v>77208</v>
       </c>
@@ -1159,10 +1119,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>zeaxanthin</t>
-        </is>
+      <c r="A22" t="str">
+        <v>zeaxanthin</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>2</v>
@@ -1176,12 +1134,12 @@
       <c r="E22" s="3" t="n">
         <v>0.9305308958112057</v>
       </c>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
       <c r="H22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="5" t="inlineStr"/>
+      <c r="I22" s="5"/>
       <c r="J22" s="2" t="n">
         <v>781129</v>
       </c>
@@ -1190,10 +1148,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>vitamin_b3</t>
-        </is>
+      <c r="A23" t="str">
+        <v>vitamin_b3</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>1</v>
@@ -1207,10 +1163,10 @@
       <c r="E23" s="3" t="n">
         <v>1.069610736564642</v>
       </c>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="5"/>
       <c r="J23" s="2" t="n">
         <v>2301</v>
       </c>
@@ -1219,10 +1175,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>vitamin_d</t>
-        </is>
+      <c r="A24" t="str">
+        <v>vitamin_d</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>12</v>
@@ -1243,7 +1197,7 @@
         <v>2.100374051179731</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>83.51000000000001</v>
+        <v>83.51</v>
       </c>
       <c r="I24" s="5" t="n">
         <v>0.8427071206594762</v>
@@ -1256,10 +1210,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>vitamin_b2</t>
-        </is>
+      <c r="A25" t="str">
+        <v>vitamin_b2</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>3</v>
@@ -1293,10 +1245,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>lycopene</t>
-        </is>
+      <c r="A26" t="str">
+        <v>lycopene</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>3</v>
@@ -1330,10 +1280,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>calcium</t>
-        </is>
+      <c r="A27" t="str">
+        <v>calcium</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>4</v>
@@ -1367,10 +1315,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>total_dietary_fiber_intake</t>
-        </is>
+      <c r="A28" t="str">
+        <v>total_dietary_fiber_intake</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>3</v>
@@ -1404,10 +1350,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>insoluble_dietary_fiber_intake</t>
-        </is>
+      <c r="A29" t="str">
+        <v>insoluble_dietary_fiber_intake</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>1</v>
@@ -1421,10 +1365,10 @@
       <c r="E29" s="3" t="n">
         <v>1.049727123434263</v>
       </c>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="5" t="inlineStr"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="5"/>
       <c r="J29" s="2" t="n">
         <v>2301</v>
       </c>
@@ -1433,10 +1377,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>choline</t>
-        </is>
+      <c r="A30" t="str">
+        <v>choline</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>2</v>
@@ -1450,12 +1392,12 @@
       <c r="E30" s="3" t="n">
         <v>1.059609029509115</v>
       </c>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
       <c r="H30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="5" t="inlineStr"/>
+      <c r="I30" s="5"/>
       <c r="J30" s="2" t="n">
         <v>568979</v>
       </c>
@@ -1464,10 +1406,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>animal_protein_intake</t>
-        </is>
+      <c r="A31" t="str">
+        <v>animal_protein_intake</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>1</v>
@@ -1481,10 +1421,10 @@
       <c r="E31" s="3" t="n">
         <v>1.28</v>
       </c>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="5" t="inlineStr"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="5"/>
       <c r="J31" s="2" t="n">
         <v>774952</v>
       </c>
@@ -1493,10 +1433,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>vitamin_b1</t>
-        </is>
+      <c r="A32" t="str">
+        <v>vitamin_b1</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>2</v>
@@ -1510,12 +1448,12 @@
       <c r="E32" s="3" t="n">
         <v>2.234907857172984</v>
       </c>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
       <c r="H32" s="4" t="n">
-        <v>85.51000000000001</v>
-      </c>
-      <c r="I32" s="5" t="inlineStr"/>
+        <v>85.51</v>
+      </c>
+      <c r="I32" s="5"/>
       <c r="J32" s="2" t="n">
         <v>4597</v>
       </c>
@@ -1524,10 +1462,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>monounsaturated_fat_mufa</t>
-        </is>
+      <c r="A33" t="str">
+        <v>monounsaturated_fat_mufa</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>1</v>
@@ -1541,10 +1477,10 @@
       <c r="E33" s="3" t="n">
         <v>1.32</v>
       </c>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="5" t="inlineStr"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="5"/>
       <c r="J33" s="2" t="n">
         <v>774952</v>
       </c>
@@ -1553,10 +1489,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>polyunsaturated_fat_pufa</t>
-        </is>
+      <c r="A34" t="str">
+        <v>polyunsaturated_fat_pufa</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>1</v>
@@ -1570,10 +1504,10 @@
       <c r="E34" s="3" t="n">
         <v>1.31</v>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="5" t="inlineStr"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="5"/>
       <c r="J34" s="2" t="n">
         <v>774952</v>
       </c>
@@ -1582,10 +1516,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>sugar_sweetened_beverage_intake</t>
-        </is>
+      <c r="A35" t="str">
+        <v>sugar_sweetened_beverage_intake</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>4</v>
@@ -1619,10 +1551,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>processed_meat_intake</t>
-        </is>
+      <c r="A36" t="str">
+        <v>processed_meat_intake</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>6</v>
@@ -1643,7 +1573,7 @@
         <v>2.09765466731294</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>77.04000000000001</v>
+        <v>77.04</v>
       </c>
       <c r="I36" s="5" t="n">
         <v>0.009426052809354803</v>
@@ -1656,10 +1586,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ultra_processed_food_intake</t>
-        </is>
+      <c r="A37" t="str">
+        <v>ultra_processed_food_intake</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>3</v>
@@ -1693,10 +1621,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>vitamin_a</t>
-        </is>
+      <c r="A38" t="str">
+        <v>vitamin_a</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>2</v>
@@ -1710,12 +1636,12 @@
       <c r="E38" s="3" t="n">
         <v>2.844820578397655</v>
       </c>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
       <c r="H38" s="4" t="n">
-        <v>92.65000000000001</v>
-      </c>
-      <c r="I38" s="5" t="inlineStr"/>
+        <v>92.65</v>
+      </c>
+      <c r="I38" s="5"/>
       <c r="J38" s="2" t="n">
         <v>4597</v>
       </c>
@@ -1724,10 +1650,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>manganese</t>
-        </is>
+      <c r="A39" t="str">
+        <v>manganese</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>1</v>
@@ -1741,10 +1665,10 @@
       <c r="E39" s="3" t="n">
         <v>1.905481103347211</v>
       </c>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="5" t="inlineStr"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="5"/>
       <c r="J39" s="2" t="n">
         <v>61321</v>
       </c>
@@ -1753,10 +1677,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>non_nutritive_sweetener_intake</t>
-        </is>
+      <c r="A40" t="str">
+        <v>non_nutritive_sweetener_intake</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>2</v>
@@ -1770,12 +1692,12 @@
       <c r="E40" s="3" t="n">
         <v>1.633459241320152</v>
       </c>
-      <c r="F40" s="3" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
       <c r="H40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="5" t="inlineStr"/>
+      <c r="I40" s="5"/>
       <c r="J40" s="2" t="n">
         <v>115981</v>
       </c>
@@ -1784,10 +1706,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>potassium</t>
-        </is>
+      <c r="A41" t="str">
+        <v>potassium</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>1</v>
@@ -1801,10 +1721,10 @@
       <c r="E41" s="3" t="n">
         <v>1.895554083552581</v>
       </c>
-      <c r="F41" s="3" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="5" t="inlineStr"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="5"/>
       <c r="J41" s="2" t="n">
         <v>120852</v>
       </c>
@@ -1813,10 +1733,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>dietary_protein_intake</t>
-        </is>
+      <c r="A42" t="str">
+        <v>dietary_protein_intake</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>2</v>
@@ -1830,12 +1748,12 @@
       <c r="E42" s="3" t="n">
         <v>2.242071017259514</v>
       </c>
-      <c r="F42" s="3" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
       <c r="H42" s="4" t="n">
-        <v>66.45999999999999</v>
-      </c>
-      <c r="I42" s="5" t="inlineStr"/>
+        <v>66.46</v>
+      </c>
+      <c r="I42" s="5"/>
       <c r="J42" s="2" t="n">
         <v>776349</v>
       </c>
@@ -1844,10 +1762,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>yogurt</t>
-        </is>
+      <c r="A43" t="str">
+        <v>yogurt</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>1</v>
@@ -1861,10 +1777,10 @@
       <c r="E43" s="3" t="n">
         <v>1.664203031653749</v>
       </c>
-      <c r="F43" s="3" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="5" t="inlineStr"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="5"/>
       <c r="J43" s="2" t="n">
         <v>1812</v>
       </c>
@@ -1873,10 +1789,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>red_meat</t>
-        </is>
+      <c r="A44" t="str">
+        <v>red_meat</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>6</v>
@@ -1910,10 +1824,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>docosahexaenoic_acid</t>
-        </is>
+      <c r="A45" t="str">
+        <v>docosahexaenoic_acid</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>1</v>
@@ -1927,10 +1839,10 @@
       <c r="E45" s="3" t="n">
         <v>2.26250941134674</v>
       </c>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="5"/>
       <c r="J45" s="2" t="n">
         <v>84063</v>
       </c>
@@ -1939,10 +1851,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>omega_3_fatty_acids</t>
-        </is>
+      <c r="A46" t="str">
+        <v>omega_3_fatty_acids</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>1</v>
@@ -1956,10 +1866,10 @@
       <c r="E46" s="3" t="n">
         <v>2.27241730386655</v>
       </c>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="5" t="inlineStr"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="5"/>
       <c r="J46" s="2" t="n">
         <v>84063</v>
       </c>
@@ -1968,10 +1878,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
+      <c r="A47" t="str">
+        <v>dairy</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>6</v>
@@ -2005,10 +1913,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>zinc</t>
-        </is>
+      <c r="A48" t="str">
+        <v>zinc</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>1</v>
@@ -2022,10 +1928,10 @@
       <c r="E48" s="3" t="n">
         <v>2.954816153625951</v>
       </c>
-      <c r="F48" s="3" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="5" t="inlineStr"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="5"/>
       <c r="J48" s="2" t="n">
         <v>63257</v>
       </c>
@@ -2034,10 +1940,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>oleic_acid</t>
-        </is>
+      <c r="A49" t="str">
+        <v>oleic_acid</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>1</v>
@@ -2051,10 +1955,10 @@
       <c r="E49" s="3" t="n">
         <v>2.871633714999859</v>
       </c>
-      <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="5" t="inlineStr"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="5"/>
       <c r="J49" s="2" t="n">
         <v>2143</v>
       </c>
@@ -2063,10 +1967,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>carnitine</t>
-        </is>
+      <c r="A50" t="str">
+        <v>carnitine</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>1</v>
@@ -2080,10 +1982,10 @@
       <c r="E50" s="3" t="n">
         <v>3.871032294091838</v>
       </c>
-      <c r="F50" s="3" t="inlineStr"/>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="5" t="inlineStr"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="5"/>
       <c r="J50" s="2" t="n">
         <v>534</v>
       </c>
@@ -2092,10 +1994,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>copper</t>
-        </is>
+      <c r="A51" t="str">
+        <v>copper</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>2</v>
@@ -2109,12 +2009,12 @@
       <c r="E51" s="3" t="n">
         <v>13.83774495311215</v>
       </c>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
       <c r="H51" s="4" t="n">
-        <v>86.43000000000001</v>
-      </c>
-      <c r="I51" s="5" t="inlineStr"/>
+        <v>86.43</v>
+      </c>
+      <c r="I51" s="5"/>
       <c r="J51" s="2" t="n">
         <v>95958</v>
       </c>

</xml_diff>